<commit_message>
feat: add course materials and quizzes for databases and robot factory lessons
</commit_message>
<xml_diff>
--- a/3d-school-start/lesson-05/quiz.xlsx
+++ b/3d-school-start/lesson-05/quiz.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Kahoot" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -11,8 +11,8 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <fonts count="1">
     <font>
+      <name val="Calibri"/>
       <sz val="11"/>
-      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="2">
@@ -32,8 +32,11 @@
       <diagonal/>
     </border>
   </borders>
+  <cellStyleXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
 </styleSheet>
 </file>
@@ -81,12 +84,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Ce primeau campionii la Jocurile Olimpice din Grecia antica?</t>
+          <t>Ce primeau campionii la Jocurile Olimpice din Grecia antică?</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Cununa de maslin</t>
+          <t>Cunună de măslin</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -96,7 +99,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>O cupa mare</t>
+          <t>O cupă mare</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -107,24 +110,26 @@
       <c r="F2">
         <v>20</v>
       </c>
-      <c r="G2">
-        <v>1</v>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Cu ce instrument se taia ramura sacra de maslin in Grecia antica?</t>
+          <t>Cu ce instrument se tăia ramura sacră de măslin în Grecia antică?</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Foarfeca de aur</t>
+          <t>Foarfecă de aur</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Cutit de piatra</t>
+          <t>Cuțit de piatră</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -140,14 +145,16 @@
       <c r="F3">
         <v>20</v>
       </c>
-      <c r="G3">
-        <v>1</v>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Cine a batut primele discuri metalice de onoare numite medalioane?</t>
+          <t>Cine a bătut primele discuri metalice de onoare numite medalioane?</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -157,7 +164,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Piratii antici</t>
+          <t>Pirații antici</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -173,14 +180,16 @@
       <c r="F4">
         <v>20</v>
       </c>
-      <c r="G4">
-        <v>1</v>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Ce artist din Renastere a transformat medalia intr-o opera de arta?</t>
+          <t>Ce artist din Renaștere a transformat medalia într-o operă de artă?</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -206,14 +215,16 @@
       <c r="F5">
         <v>20</v>
       </c>
-      <c r="G5">
-        <v>1</v>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Ce medalie primea invingatorul la primele Jocuri Olimpice moderne?</t>
+          <t>Ce medalie primea învingătorul la primele Jocuri Olimpice moderne (1896)?</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -228,7 +239,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Medalie de platina</t>
+          <t>Medalie de platină</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -239,14 +250,16 @@
       <c r="F6">
         <v>20</v>
       </c>
-      <c r="G6">
-        <v>1</v>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Ce a primit sportivul de pe locul al treilea la Atena in 1896?</t>
+          <t>Ce a primit sportivul de pe locul al treilea la Atena în 1896?</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -261,25 +274,27 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>O insigna</t>
+          <t>O insignă</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>O cupa</t>
+          <t>O cupă</t>
         </is>
       </c>
       <c r="F7">
         <v>20</v>
       </c>
-      <c r="G7">
-        <v>1</v>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>In ce an si oras a aparut oficial trio-ul Aur, Argint si Bronz?</t>
+          <t>În ce an și oraș a apărut oficial trio-ul Aur, Argint și Bronz?</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -305,24 +320,26 @@
       <c r="F8">
         <v>20</v>
       </c>
-      <c r="G8">
-        <v>1</v>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>De ce a fost ales aurul pentru locul intai?</t>
+          <t>De ce a fost ales aurul pentru locul întâi?</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Nu rugineste deloc</t>
+          <t>Nu ruginește niciodată</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Este foarte usor</t>
+          <t>Este foarte ușor</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -338,8 +355,10 @@
       <c r="F9">
         <v>20</v>
       </c>
-      <c r="G9">
-        <v>1</v>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
     </row>
     <row r="10">
@@ -350,35 +369,37 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Cupru si cositor</t>
+          <t>Cupru și cositor</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Fier si nisip</t>
+          <t>Fier și nisip</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Aluminiu si argint</t>
+          <t>Aluminiu și argint</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Plumb si aur</t>
+          <t>Plumb și aur</t>
         </is>
       </c>
       <c r="F10">
         <v>20</v>
       </c>
-      <c r="G10">
-        <v>1</v>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>La ce editie a Jocurilor Olimpice a aparut prima data panglica de gat?</t>
+          <t>La ce ediție a Jocurilor Olimpice a apărut prima dată panglica de gât?</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -404,62 +425,66 @@
       <c r="F11">
         <v>20</v>
       </c>
-      <c r="G11">
-        <v>1</v>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Ce simbolizeaza crenguta de dafin sculptata pe marginea medaliilor?</t>
+          <t>Ce simbolizează crenguța de dafin (laur) sculptată pe marginea medaliilor?</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Victoria eterna</t>
+          <t>Victoria eternă</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Noaptea linistita</t>
+          <t>Noaptea liniștită</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Viteza vantului</t>
+          <t>Viteza vântului</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Apa marii</t>
+          <t>Apa mării</t>
         </is>
       </c>
       <c r="F12">
         <v>20</v>
       </c>
-      <c r="G12">
-        <v>1</v>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Cine merita o medalie de aur in viata noastra de zi cu zi?</t>
+          <t>Cine merită o medalie de aur în viața noastră de zi cu zi?</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Oamenii dragi noua</t>
+          <t>Oamenii dragi nouă</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Doar extraterestrii</t>
+          <t>Doar extratereștrii</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Numai robotii</t>
+          <t>Numai roboții</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -470,8 +495,10 @@
       <c r="F13">
         <v>20</v>
       </c>
-      <c r="G13">
-        <v>1</v>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>